<commit_message>
docs(question-bank): sync workflow v4 packages and Review preflight
</commit_message>
<xml_diff>
--- a/docs/question-bank/templates/O2I_Question_Bank_Import_Template.xlsx
+++ b/docs/question-bank/templates/O2I_Question_Bank_Import_Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R27a0977fbe684cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R5b7f80b062604738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="Rd0bb0d280f614fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" r:id="R4b74d41619c74aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rb2076f06d15141ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R0a4d52eb25c74d56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -709,10 +709,10 @@
         <x:v>审核</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>最终批准</x:v>
+        <x:v>后台发布确认</x:v>
       </x:c>
       <x:c r="C12" s="25" t="str">
-        <x:v>只有授权人工审核人在数学、来源/权利、分类和渲染四个关卡全部通过后，才可手动设置 approved。</x:v>
+        <x:v>v4导出五项审核pending，reviewed_by/at空；人工决定另存，后台核对内容/答案/显示/标签后确认一次。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
@@ -833,7 +833,7 @@
         <x:v>推断字段</x:v>
       </x:c>
       <x:c r="C23" s="25" t="str">
-        <x:v>难度、课程范围、主题、技能、表示方式、计算器政策、误区与 AI 草拟解答属于推断，写入 ai_inference_notes 并添加 ai_flags。</x:v>
+        <x:v>AI建议写ai_inference_notes；flags记录来源性质或真实未解决问题，不机械给全批加相同uncertain。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
@@ -888,7 +888,7 @@
         <x:v>配套文档</x:v>
       </x:c>
       <x:c r="C28" s="27" t="str">
-        <x:v>参见 O2I_AI_QUESTION_WORKFLOW_ZH.md、O2I_HUMAN_REVIEW_SOP_ZH.md、O2I_QUESTION_IMPORT_SCHEMA.md 和 O2I_QUESTION_PROCESSING_PROMPT_ZH.md。</x:v>
+        <x:v>当前使用O2I_AI_PRACTICE_WORKFLOW_V4_ZH.md、SOP、Schema、O2I_CED_CODE_REFERENCE.md；不要混用旧ZIP。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>